<commit_message>
Add .gitattributes to normalize line endings
</commit_message>
<xml_diff>
--- a/week-02/events_sample.xlsx
+++ b/week-02/events_sample.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sthef\data-analytics\week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9988EDAE-5040-4432-9022-A8C0C7E1BCD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D68AB8-19BF-4FA0-A417-469AE6789DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4092" yWindow="1776" windowWidth="17040" windowHeight="8916" xr2:uid="{ACA9E12C-C974-49B2-99BE-524182F6A9AE}"/>
+    <workbookView xWindow="2260" yWindow="670" windowWidth="16940" windowHeight="8900" xr2:uid="{ACA9E12C-C974-49B2-99BE-524182F6A9AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -263,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -282,7 +281,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -292,7 +290,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,17 +624,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8398B12-CCD7-465B-A5C6-DBDC8B28AA2B}">
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="16.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L66"/>
+  <sheetFormatPr defaultColWidth="16.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" style="5"/>
+    <col min="1" max="1" width="11.36328125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="16.08984375" style="5"/>
     <col min="8" max="8" width="16" style="5" customWidth="1"/>
-    <col min="9" max="9" width="16.109375" style="5"/>
-    <col min="11" max="11" width="19.21875" customWidth="1"/>
+    <col min="9" max="9" width="16.08984375" style="5"/>
+    <col min="11" max="11" width="19.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>32</v>
       </c>
@@ -665,7 +662,7 @@
       <c r="I1" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="10" t="s">
         <v>33</v>
       </c>
       <c r="K1" s="8" t="s">
@@ -675,7 +672,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -709,11 +706,11 @@
       <c r="K2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -747,11 +744,11 @@
       <c r="K3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -785,11 +782,11 @@
       <c r="K4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>2</v>
       </c>
@@ -823,11 +820,11 @@
       <c r="K5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>2</v>
       </c>
@@ -861,11 +858,11 @@
       <c r="K6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>2</v>
       </c>
@@ -899,11 +896,11 @@
       <c r="K7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -937,11 +934,11 @@
       <c r="K8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>3</v>
       </c>
@@ -975,11 +972,11 @@
       <c r="K9" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>4</v>
       </c>
@@ -1013,11 +1010,11 @@
       <c r="K10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="10" t="s">
+      <c r="L10" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>4</v>
       </c>
@@ -1051,444 +1048,564 @@
       <c r="K11" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="10" t="s">
+      <c r="L11" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5668F06-A0B0-487A-AD25-06F446AE0083}">
-  <dimension ref="A3:I29"/>
-  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14"/>
+      <c r="E14"/>
+      <c r="H14"/>
+      <c r="I14"/>
+    </row>
+    <row r="15" spans="1:12" ht="16" x14ac:dyDescent="0.4">
+      <c r="A15" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="E15"/>
+      <c r="F15" s="14" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="H15"/>
+      <c r="I15"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A16" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="E16"/>
+      <c r="F16" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I16" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="4">
+      <c r="C17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17"/>
+      <c r="F17" s="4">
         <v>101</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="4">
+      <c r="G17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I17" s="4">
         <v>500</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
         <v>1</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" s="4">
+      <c r="C18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18"/>
+      <c r="F18" s="4">
         <v>101</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I6" s="4">
+      <c r="G18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I18" s="4">
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
         <v>1</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F7" s="4">
+      <c r="C19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19"/>
+      <c r="F19" s="4">
         <v>101</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I7" s="4">
+      <c r="G19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I19" s="4">
         <v>500</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
-        <v>2</v>
-      </c>
-      <c r="B8" s="2" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>2</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="4">
+      <c r="E20"/>
+      <c r="F20" s="4">
         <v>102</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="4">
+      <c r="H20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I20" s="4">
         <v>1200</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>2</v>
-      </c>
-      <c r="B9" s="2" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>2</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="4">
+      <c r="E21"/>
+      <c r="F21" s="4">
         <v>102</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I9" s="4">
+      <c r="H21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="4">
         <v>1200</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
-        <v>2</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>2</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="4">
+      <c r="E22"/>
+      <c r="F22" s="4">
         <v>102</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I10" s="4">
+      <c r="H22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="4">
         <v>1200</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>3</v>
-      </c>
-      <c r="B11" s="2" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>3</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="4">
+      <c r="E23"/>
+      <c r="F23" s="4">
         <v>103</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I23" s="4">
         <v>5000</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
-        <v>3</v>
-      </c>
-      <c r="B12" s="2" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>3</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="4">
+      <c r="E24"/>
+      <c r="F24" s="4">
         <v>103</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="4">
+      <c r="I24" s="4">
         <v>5000</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
         <v>4</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="4">
+      <c r="E25"/>
+      <c r="F25" s="4">
         <v>104</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="4">
+      <c r="H25" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I25" s="4">
         <v>3000</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="4">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
         <v>4</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="4">
+      <c r="E26"/>
+      <c r="F26" s="4">
         <v>104</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I14" s="4">
+      <c r="H26" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I26" s="4">
         <v>3000</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="15" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27"/>
+      <c r="E27"/>
+      <c r="H27"/>
+      <c r="I27"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28"/>
+      <c r="E28"/>
+      <c r="H28"/>
+      <c r="I28"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29"/>
+      <c r="E29"/>
+      <c r="H29"/>
+      <c r="I29"/>
+    </row>
+    <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.4">
+      <c r="A30" s="14" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+      <c r="E30"/>
+      <c r="H30"/>
+      <c r="I30"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B31" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C31" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D31" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F19" s="16"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="4">
+      <c r="E31"/>
+      <c r="H31"/>
+      <c r="I31"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="4">
         <v>201</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C32" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D32" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="4">
+      <c r="E32"/>
+      <c r="H32"/>
+      <c r="I32"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="4">
         <v>201</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C33" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D33" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="4">
+      <c r="E33"/>
+      <c r="H33"/>
+      <c r="I33"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="4">
         <v>201</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B34" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C34" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D34" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="4">
+      <c r="E34"/>
+      <c r="H34"/>
+      <c r="I34"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="4">
         <v>202</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B35" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C35" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D35" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="4">
+      <c r="E35"/>
+      <c r="H35"/>
+      <c r="I35"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="4">
         <v>202</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B36" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C36" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D36" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="4">
+      <c r="E36"/>
+      <c r="H36"/>
+      <c r="I36"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" s="4">
         <v>202</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C37" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D37" s="9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="4">
+      <c r="E37"/>
+      <c r="H37"/>
+      <c r="I37"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" s="4">
         <v>201</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B38" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C38" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D38" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="4">
+      <c r="E38"/>
+      <c r="H38"/>
+      <c r="I38"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
         <v>201</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B39" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D39" s="9" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="4">
+      <c r="E39"/>
+      <c r="H39"/>
+      <c r="I39"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="4">
         <v>203</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C40" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D40" s="9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="4">
+      <c r="E40"/>
+      <c r="H40"/>
+      <c r="I40"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="4">
         <v>203</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C41" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D41" s="9" t="s">
         <v>23</v>
       </c>
-    </row>
+      <c r="E41"/>
+      <c r="H41"/>
+      <c r="I41"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42"/>
+      <c r="E42"/>
+      <c r="H42"/>
+      <c r="I42"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43"/>
+      <c r="E43"/>
+      <c r="H43"/>
+      <c r="I43"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44"/>
+      <c r="E44"/>
+      <c r="H44"/>
+      <c r="I44"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45"/>
+      <c r="E45"/>
+      <c r="H45"/>
+      <c r="I45"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46"/>
+      <c r="E46"/>
+      <c r="H46"/>
+      <c r="I46"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47"/>
+      <c r="E47"/>
+      <c r="H47"/>
+      <c r="I47"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48"/>
+      <c r="E48"/>
+      <c r="H48"/>
+      <c r="I48"/>
+    </row>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>